<commit_message>
Kit Médicos: rotina 12/18 na planilha 03, crédito à vista na conciliação 16, NUMEROS.md e manual alinhados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-medicos/03-rotina-da-semana.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-medicos/03-rotina-da-semana.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Em Rotina, ajuste as linhas: dia, rotina, minutos e responsável. O exemplo soma 30 minutos por semana (15 na segunda, 15 na sexta), a maior parte com a recepção; mantenha curto, o que é longo não vira hábito.</t>
+          <t>Em Rotina, ajuste as linhas: dia, rotina, minutos e responsável. O exemplo soma 30 minutos por semana (12 na segunda, 18 na sexta), a maior parte com a recepção; mantenha curto, o que é longo não vira hábito.</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C9" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A9,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D9" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A9))</f>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C13" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A13,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D13" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A13))</f>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="F17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$34:$BD$34,($K$4-7)))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G17" s="26" t="str">
         <f>IF(E17="","",REPT("█",ROUND(E17*10,0)))</f>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="F18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$34:$BD$34,($K$4-6)))</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G18" s="26" t="str">
         <f>IF(E18="","",REPT("█",ROUND(E18*10,0)))</f>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$34:$BD$34,($K$4-5)))</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G19" s="26" t="str">
         <f>IF(E19="","",REPT("█",ROUND(E19*10,0)))</f>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="F20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$34:$BD$34,($K$4-4)))</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G20" s="26" t="str">
         <f>IF(E20="","",REPT("█",ROUND(E20*10,0)))</f>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$34:$BD$34,($K$4-3)))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G21" s="26" t="str">
         <f>IF(E21="","",REPT("█",ROUND(E21*10,0)))</f>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$34:$BD$34,($K$4-2)))</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G22" s="26" t="str">
         <f>IF(E22="","",REPT("█",ROUND(E22*10,0)))</f>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="F24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$34:$BD$34,($K$4-0)))</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G24" s="26" t="str">
         <f>IF(E24="","",REPT("█",ROUND(E24*10,0)))</f>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="C30" s="22">
         <f>IF(Rotina!$B6="","",Rotina!$C6)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="22" t="str">
         <f>IF(Rotina!$B6="","",Rotina!$D6)</f>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C31" s="22">
         <f>IF(Rotina!$B7="","",Rotina!$C7)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="22" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$D7)</f>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C32" s="22">
         <f>IF(Rotina!$B8="","",Rotina!$C8)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" s="22" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$D8)</f>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C34" s="22">
         <f>IF(Rotina!$B10="","",Rotina!$C10)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" s="22" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$D10)</f>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="C36" s="22">
         <f>IF(Rotina!$B12="","",Rotina!$C12)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" s="22" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$D12)</f>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="C37" s="22">
         <f>IF(Rotina!$B13="","",Rotina!$C13)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D37" s="22" t="str">
         <f>IF(Rotina!$B13="","",Rotina!$D13)</f>
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="C6" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="36" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="C7" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="C8" s="36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
@@ -3864,7 +3864,7 @@
         </is>
       </c>
       <c r="C10" s="36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="C12" s="36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
@@ -4176,7 +4176,7 @@
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="36" t="inlineStr">
         <is>
@@ -6118,27 +6118,27 @@
       </c>
       <c r="AG34" s="37">
         <f>SUMIF(AG5:AG28,"Sim",$C$5:$C$28)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AH34" s="37">
         <f>SUMIF(AH5:AH28,"Sim",$C$5:$C$28)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AI34" s="37">
         <f>SUMIF(AI5:AI28,"Sim",$C$5:$C$28)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AJ34" s="37">
         <f>SUMIF(AJ5:AJ28,"Sim",$C$5:$C$28)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AK34" s="37">
         <f>SUMIF(AK5:AK28,"Sim",$C$5:$C$28)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AL34" s="37">
         <f>SUMIF(AL5:AL28,"Sim",$C$5:$C$28)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AM34" s="37">
         <f>SUMIF(AM5:AM28,"Sim",$C$5:$C$28)</f>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="AN34" s="37">
         <f>SUMIF(AN5:AN28,"Sim",$C$5:$C$28)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AO34" s="37">
         <f>SUMIF(AO5:AO28,"Sim",$C$5:$C$28)</f>

</xml_diff>

<commit_message>
Kit Medicos: revisao interna das planilhas aplicada (25 achados) - cabecalho da 08, orcamentos coerentes, agenda com folga de 12 meses, provisao no DRE, repasse sem cobranca dupla, rotina 12/18, regras escritas; 677 verificacoes de coerencia OK
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-medicos/03-rotina-da-semana.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-medicos/03-rotina-da-semana.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Em Rotina, ajuste as linhas: dia, rotina, minutos e responsável. O exemplo soma 30 minutos por semana (12 na segunda, 18 na sexta), a maior parte com a recepção; mantenha curto, o que é longo não vira hábito.</t>
+          <t>Em Rotina, ajuste as linhas: dia, rotina, minutos e responsável. O exemplo soma 30 minutos por semana (3 rotinas de segunda = 12 min; 5 de sexta = 18 min), a maior parte com a recepção; mantenha curto, o que é longo não vira hábito. O checklist do dia (04) é da recepção e corre por fora destes 30 minutos.</t>
         </is>
       </c>
     </row>
@@ -955,8 +955,8 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="3" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="26" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1011,7 +1011,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="15">
         <f>IF(OR($K$4=0,$K$7=0),"",SUMPRODUCT((Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)*Rotina!$E$30:$BD$30)/($K$6*$K$7))</f>
-        <v>0.833333333333333</v>
+        <v>0.84375</v>
       </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="16" t="str">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="K7" s="14">
         <f>COUNTA(Rotina!$B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B9" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A9,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A9,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
@@ -1118,11 +1118,11 @@
       </c>
       <c r="E9" s="22">
         <f>IF($K$4=0,"",B9*$K$6)</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F9" s="23">
         <f>IF(OR(E9="",E9=0),"",D9/E9)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D13" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A13))</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E13" s="22">
         <f>IF($K$4=0,"",B13*$K$6)</f>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="F13" s="23">
         <f>IF(OR(E13="",E13=0),"",D13/E13)</f>
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="14"/>
@@ -1289,23 +1289,23 @@
       </c>
       <c r="C17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$30:$BD$30,($K$4-7)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$32:$BD$32,($K$4-7)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" s="23">
         <f>IF(OR(A17="",D17=0),"",C17/D17)</f>
-        <v>0.555555555555556</v>
+        <v>0.5</v>
       </c>
       <c r="F17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$34:$BD$34,($K$4-7)))</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G17" s="26" t="str">
         <f>IF(E17="","",REPT("█",ROUND(E17*10,0)))</f>
-        <v>██████</v>
+        <v>█████</v>
       </c>
       <c r="H17" s="27" t="n"/>
     </row>
@@ -1320,19 +1320,19 @@
       </c>
       <c r="C18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$30:$BD$30,($K$4-6)))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$32:$BD$32,($K$4-6)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="23">
         <f>IF(OR(A18="",D18=0),"",C18/D18)</f>
-        <v>0.888888888888889</v>
+        <v>0.875</v>
       </c>
       <c r="F18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$34:$BD$34,($K$4-6)))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G18" s="26" t="str">
         <f>IF(E18="","",REPT("█",ROUND(E18*10,0)))</f>
@@ -1351,23 +1351,23 @@
       </c>
       <c r="C19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$30:$BD$30,($K$4-5)))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$32:$BD$32,($K$4-5)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="23">
         <f>IF(OR(A19="",D19=0),"",C19/D19)</f>
-        <v>0.888888888888889</v>
+        <v>0.75</v>
       </c>
       <c r="F19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$34:$BD$34,($K$4-5)))</f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G19" s="26" t="str">
         <f>IF(E19="","",REPT("█",ROUND(E19*10,0)))</f>
-        <v>█████████</v>
+        <v>████████</v>
       </c>
       <c r="H19" s="27" t="n"/>
     </row>
@@ -1386,19 +1386,19 @@
       </c>
       <c r="D20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$32:$BD$32,($K$4-4)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" s="23">
         <f>IF(OR(A20="",D20=0),"",C20/D20)</f>
-        <v>0.888888888888889</v>
+        <v>1</v>
       </c>
       <c r="F20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$34:$BD$34,($K$4-4)))</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G20" s="26" t="str">
         <f>IF(E20="","",REPT("█",ROUND(E20*10,0)))</f>
-        <v>█████████</v>
+        <v>██████████</v>
       </c>
       <c r="H20" s="27" t="n"/>
     </row>
@@ -1413,23 +1413,23 @@
       </c>
       <c r="C21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$30:$BD$30,($K$4-3)))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$32:$BD$32,($K$4-3)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="23">
         <f>IF(OR(A21="",D21=0),"",C21/D21)</f>
-        <v>0.888888888888889</v>
+        <v>0.75</v>
       </c>
       <c r="F21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$34:$BD$34,($K$4-3)))</f>
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G21" s="26" t="str">
         <f>IF(E21="","",REPT("█",ROUND(E21*10,0)))</f>
-        <v>█████████</v>
+        <v>████████</v>
       </c>
       <c r="H21" s="27" t="n"/>
     </row>
@@ -1448,19 +1448,19 @@
       </c>
       <c r="D22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$32:$BD$32,($K$4-2)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="23">
         <f>IF(OR(A22="",D22=0),"",C22/D22)</f>
-        <v>0.777777777777778</v>
+        <v>0.875</v>
       </c>
       <c r="F22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$34:$BD$34,($K$4-2)))</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G22" s="26" t="str">
         <f>IF(E22="","",REPT("█",ROUND(E22*10,0)))</f>
-        <v>████████</v>
+        <v>█████████</v>
       </c>
       <c r="H22" s="27" t="n"/>
     </row>
@@ -1479,19 +1479,19 @@
       </c>
       <c r="D23" s="22">
         <f>IF(A23="","",INDEX(Rotina!$E$32:$BD$32,($K$4-1)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="23">
         <f>IF(OR(A23="",D23=0),"",C23/D23)</f>
-        <v>0.777777777777778</v>
+        <v>0.875</v>
       </c>
       <c r="F23" s="22">
         <f>IF(A23="","",INDEX(Rotina!$E$34:$BD$34,($K$4-1)))</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G23" s="26" t="str">
         <f>IF(E23="","",REPT("█",ROUND(E23*10,0)))</f>
-        <v>████████</v>
+        <v>█████████</v>
       </c>
       <c r="H23" s="27" t="n"/>
     </row>
@@ -1506,19 +1506,19 @@
       </c>
       <c r="C24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$30:$BD$30,($K$4-0)))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$32:$BD$32,($K$4-0)))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="23">
         <f>IF(OR(A24="",D24=0),"",C24/D24)</f>
-        <v>0.888888888888889</v>
+        <v>0.875</v>
       </c>
       <c r="F24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$34:$BD$34,($K$4-0)))</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G24" s="26" t="str">
         <f>IF(E24="","",REPT("█",ROUND(E24*10,0)))</f>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="C30" s="22">
         <f>IF(Rotina!$B6="","",Rotina!$C6)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="22" t="str">
         <f>IF(Rotina!$B6="","",Rotina!$D6)</f>
@@ -1658,11 +1658,11 @@
       </c>
       <c r="B31" s="21" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$B7)</f>
-        <v>Ligar ou mandar mensagem para a lista de retorno (02)</v>
+        <v>Ligar para a lista de retorno (02) e registrar as faltas da semana passada</v>
       </c>
       <c r="C31" s="22">
         <f>IF(Rotina!$B7="","",Rotina!$C7)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="22" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$D7)</f>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E31" s="22">
         <f>IF(OR(Rotina!$B7="",$K$4=0),"",SUMPRODUCT((Rotina!$E$7:$BD$7="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F31" s="22">
         <f>IF(E31="","",$K$6)</f>
@@ -1678,33 +1678,33 @@
       </c>
       <c r="G31" s="23">
         <f>IF(OR(E31="",F31=0),"",E31/F31)</f>
-        <v>0.25</v>
-      </c>
-      <c r="H31" s="21" t="str">
+        <v>1</v>
+      </c>
+      <c r="H31" s="21">
         <f>IF(G31="","",IF(G31&lt;0.5,"Pulada na maioria das semanas",IF(G31&lt;0.75,"Pulada às vezes","")))</f>
-        <v>Pulada na maioria das semanas</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="22" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$A8)</f>
-        <v>Segunda</v>
+        <v>Sexta</v>
       </c>
       <c r="B32" s="21" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$B8)</f>
-        <v>Registrar as faltas da semana passada e remarcar</v>
+        <v>Conferir os fechamentos da semana no Caixa (09)</v>
       </c>
       <c r="C32" s="22">
         <f>IF(Rotina!$B8="","",Rotina!$C8)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D32" s="22" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$D8)</f>
-        <v>Bruna Carvalho</v>
+        <v>Dra. Carolina Mendes</v>
       </c>
       <c r="E32" s="22">
         <f>IF(OR(Rotina!$B8="",$K$4=0),"",SUMPRODUCT((Rotina!$E$8:$BD$8="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" s="22">
         <f>IF(E32="","",$K$6)</f>
@@ -1712,11 +1712,11 @@
       </c>
       <c r="G32" s="23">
         <f>IF(OR(E32="",F32=0),"",E32/F32)</f>
-        <v>0.75</v>
-      </c>
-      <c r="H32" s="21">
+        <v>0.5</v>
+      </c>
+      <c r="H32" s="21" t="str">
         <f>IF(G32="","",IF(G32&lt;0.5,"Pulada na maioria das semanas",IF(G32&lt;0.75,"Pulada às vezes","")))</f>
-        <v/>
+        <v>Pulada às vezes</v>
       </c>
     </row>
     <row r="33">
@@ -1726,15 +1726,15 @@
       </c>
       <c r="B33" s="21" t="str">
         <f>IF(Rotina!$B9="","",Rotina!$B9)</f>
-        <v>Lançar os fechamentos do dia da semana no Caixa (09)</v>
+        <v>Marcar parcelas recebidas e enviar a cobrança educada (14)</v>
       </c>
       <c r="C33" s="22">
         <f>IF(Rotina!$B9="","",Rotina!$C9)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="22" t="str">
         <f>IF(Rotina!$B9="","",Rotina!$D9)</f>
-        <v>Dra. Carolina Mendes</v>
+        <v>Bruna Carvalho</v>
       </c>
       <c r="E33" s="22">
         <f>IF(OR(Rotina!$B9="",$K$4=0),"",SUMPRODUCT((Rotina!$E$9:$BD$9="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
@@ -1760,11 +1760,11 @@
       </c>
       <c r="B34" s="21" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$B10)</f>
-        <v>Marcar parcelas recebidas e enviar a cobrança educada (14)</v>
+        <v>Separar as guias da semana e atualizar os lotes (13)</v>
       </c>
       <c r="C34" s="22">
         <f>IF(Rotina!$B10="","",Rotina!$C10)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34" s="22" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$D10)</f>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B35" s="21" t="str">
         <f>IF(Rotina!$B11="","",Rotina!$B11)</f>
-        <v>Separar as guias da semana e atualizar os lotes (13)</v>
+        <v>Atualizar os orçamentos apresentados e aprovados (15)</v>
       </c>
       <c r="C35" s="22">
         <f>IF(Rotina!$B11="","",Rotina!$C11)</f>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="E35" s="22">
         <f>IF(OR(Rotina!$B11="",$K$4=0),"",SUMPRODUCT((Rotina!$E$11:$BD$11="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" s="22">
         <f>IF(E35="","",$K$6)</f>
@@ -1814,11 +1814,11 @@
       </c>
       <c r="G35" s="23">
         <f>IF(OR(E35="",F35=0),"",E35/F35)</f>
-        <v>0.75</v>
-      </c>
-      <c r="H35" s="21">
+        <v>0.5</v>
+      </c>
+      <c r="H35" s="21" t="str">
         <f>IF(G35="","",IF(G35&lt;0.5,"Pulada na maioria das semanas",IF(G35&lt;0.75,"Pulada às vezes","")))</f>
-        <v/>
+        <v>Pulada às vezes</v>
       </c>
     </row>
     <row r="36">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="B36" s="21" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$B12)</f>
-        <v>Atualizar os orçamentos apresentados e aprovados (15)</v>
+        <v>Olhar o Painel da clínica (17) e anotar até 3 decisões</v>
       </c>
       <c r="C36" s="22">
         <f>IF(Rotina!$B12="","",Rotina!$C12)</f>
@@ -1836,11 +1836,11 @@
       </c>
       <c r="D36" s="22" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$D12)</f>
-        <v>Bruna Carvalho</v>
+        <v>Dr. Paulo Andrade</v>
       </c>
       <c r="E36" s="22">
         <f>IF(OR(Rotina!$B12="",$K$4=0),"",SUMPRODUCT((Rotina!$E$12:$BD$12="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F36" s="22">
         <f>IF(E36="","",$K$6)</f>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="G36" s="23">
         <f>IF(OR(E36="",F36=0),"",E36/F36)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="H36" s="21">
         <f>IF(G36="","",IF(G36&lt;0.5,"Pulada na maioria das semanas",IF(G36&lt;0.75,"Pulada às vezes","")))</f>
@@ -1856,33 +1856,33 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="str">
+      <c r="A37" s="22">
         <f>IF(Rotina!$B13="","",Rotina!$A13)</f>
-        <v>Sexta</v>
-      </c>
-      <c r="B37" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B37" s="21">
         <f>IF(Rotina!$B13="","",Rotina!$B13)</f>
-        <v>Olhar o Painel da clínica (17) e anotar até 3 decisões</v>
+        <v/>
       </c>
       <c r="C37" s="22">
         <f>IF(Rotina!$B13="","",Rotina!$C13)</f>
-        <v>3</v>
-      </c>
-      <c r="D37" s="22" t="str">
+        <v/>
+      </c>
+      <c r="D37" s="22">
         <f>IF(Rotina!$B13="","",Rotina!$D13)</f>
-        <v>Dr. Paulo Andrade</v>
+        <v/>
       </c>
       <c r="E37" s="22">
         <f>IF(OR(Rotina!$B13="",$K$4=0),"",SUMPRODUCT((Rotina!$E$13:$BD$13="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F37" s="22">
         <f>IF(E37="","",$K$6)</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="G37" s="23">
         <f>IF(OR(E37="",F37=0),"",E37/F37)</f>
-        <v>0.75</v>
+        <v/>
       </c>
       <c r="H37" s="21">
         <f>IF(G37="","",IF(G37&lt;0.5,"Pulada na maioria das semanas",IF(G37&lt;0.75,"Pulada às vezes","")))</f>
@@ -2604,7 +2604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD35"/>
+  <dimension ref="A1:BD36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="C6" s="36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="36" t="inlineStr">
         <is>
@@ -3548,11 +3548,11 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Ligar ou mandar mensagem para a lista de retorno (02)</t>
+          <t>Ligar para a lista de retorno (02) e registrar as faltas da semana passada</t>
         </is>
       </c>
       <c r="C7" s="36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
@@ -3599,27 +3599,27 @@
       </c>
       <c r="AI7" s="36" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ7" s="36" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AJ7" s="36" t="inlineStr">
+      <c r="AK7" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK7" s="36" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
       <c r="AL7" s="36" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AM7" s="36" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AN7" s="36" t="inlineStr">
@@ -3647,20 +3647,20 @@
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Sexta</t>
         </is>
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Registrar as faltas da semana passada e remarcar</t>
+          <t>Conferir os fechamentos da semana no Caixa (09)</t>
         </is>
       </c>
       <c r="C8" s="36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
-          <t>Bruna Carvalho</t>
+          <t>Dra. Carolina Mendes</t>
         </is>
       </c>
       <c r="E8" s="36" t="n"/>
@@ -3713,22 +3713,22 @@
       </c>
       <c r="AK8" s="36" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL8" s="36" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AL8" s="36" t="inlineStr">
+      <c r="AM8" s="36" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AN8" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
-        </is>
-      </c>
-      <c r="AM8" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AN8" s="36" t="inlineStr">
-        <is>
-          <t>Não</t>
         </is>
       </c>
       <c r="AO8" s="36" t="n"/>
@@ -3756,15 +3756,15 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Lançar os fechamentos do dia da semana no Caixa (09)</t>
+          <t>Marcar parcelas recebidas e enviar a cobrança educada (14)</t>
         </is>
       </c>
       <c r="C9" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="36" t="inlineStr">
         <is>
-          <t>Dra. Carolina Mendes</t>
+          <t>Bruna Carvalho</t>
         </is>
       </c>
       <c r="E9" s="36" t="n"/>
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B10" s="30" t="inlineStr">
         <is>
-          <t>Marcar parcelas recebidas e enviar a cobrança educada (14)</t>
+          <t>Separar as guias da semana e atualizar os lotes (13)</t>
         </is>
       </c>
       <c r="C10" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="36" t="inlineStr">
         <is>
@@ -3906,12 +3906,12 @@
       </c>
       <c r="AH10" s="36" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AI10" s="36" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="AJ10" s="36" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="B11" s="30" t="inlineStr">
         <is>
-          <t>Separar as guias da semana e atualizar os lotes (13)</t>
+          <t>Atualizar os orçamentos apresentados e aprovados (15)</t>
         </is>
       </c>
       <c r="C11" s="36" t="n">
@@ -4010,37 +4010,37 @@
       </c>
       <c r="AH11" s="36" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AI11" s="36" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AI11" s="36" t="inlineStr">
+      <c r="AJ11" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AJ11" s="36" t="inlineStr">
+      <c r="AK11" s="36" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AL11" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK11" s="36" t="inlineStr">
+      <c r="AM11" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AL11" s="36" t="inlineStr">
+      <c r="AN11" s="36" t="inlineStr">
         <is>
           <t>Não</t>
-        </is>
-      </c>
-      <c r="AM11" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AN11" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
         </is>
       </c>
       <c r="AO11" s="36" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>Atualizar os orçamentos apresentados e aprovados (15)</t>
+          <t>Olhar o Painel da clínica (17) e anotar até 3 decisões</t>
         </is>
       </c>
       <c r="C12" s="36" t="n">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
-          <t>Bruna Carvalho</t>
+          <t>Dr. Paulo Andrade</t>
         </is>
       </c>
       <c r="E12" s="36" t="n"/>
@@ -4119,22 +4119,22 @@
       </c>
       <c r="AI12" s="36" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ12" s="36" t="inlineStr">
+        <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AJ12" s="36" t="inlineStr">
+      <c r="AK12" s="36" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK12" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
       <c r="AL12" s="36" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AM12" s="36" t="inlineStr">
@@ -4165,24 +4165,10 @@
       <c r="BD12" s="36" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>Sexta</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Olhar o Painel da clínica (17) e anotar até 3 decisões</t>
-        </is>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>Dr. Paulo Andrade</t>
-        </is>
-      </c>
+      <c r="A13" s="36" t="n"/>
+      <c r="B13" s="30" t="n"/>
+      <c r="C13" s="36" t="n"/>
+      <c r="D13" s="36" t="n"/>
       <c r="E13" s="36" t="n"/>
       <c r="F13" s="36" t="n"/>
       <c r="G13" s="36" t="n"/>
@@ -4211,46 +4197,14 @@
       <c r="AD13" s="36" t="n"/>
       <c r="AE13" s="36" t="n"/>
       <c r="AF13" s="36" t="n"/>
-      <c r="AG13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AH13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AI13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ13" s="36" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AK13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AL13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AM13" s="36" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AN13" s="36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AG13" s="36" t="n"/>
+      <c r="AH13" s="36" t="n"/>
+      <c r="AI13" s="36" t="n"/>
+      <c r="AJ13" s="36" t="n"/>
+      <c r="AK13" s="36" t="n"/>
+      <c r="AL13" s="36" t="n"/>
+      <c r="AM13" s="36" t="n"/>
+      <c r="AN13" s="36" t="n"/>
       <c r="AO13" s="36" t="n"/>
       <c r="AP13" s="36" t="n"/>
       <c r="AQ13" s="36" t="n"/>
@@ -5258,15 +5212,15 @@
       </c>
       <c r="AG30" s="37">
         <f>COUNTIF(AG5:AG28,"Sim")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AH30" s="37">
         <f>COUNTIF(AH5:AH28,"Sim")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AI30" s="37">
         <f>COUNTIF(AI5:AI28,"Sim")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AJ30" s="37">
         <f>COUNTIF(AJ5:AJ28,"Sim")</f>
@@ -5274,7 +5228,7 @@
       </c>
       <c r="AK30" s="37">
         <f>COUNTIF(AK5:AK28,"Sim")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AL30" s="37">
         <f>COUNTIF(AL5:AL28,"Sim")</f>
@@ -5286,7 +5240,7 @@
       </c>
       <c r="AN30" s="37">
         <f>COUNTIF(AN5:AN28,"Sim")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AO30" s="37">
         <f>COUNTIF(AO5:AO28,"Sim")</f>
@@ -5473,35 +5427,35 @@
       </c>
       <c r="AG31" s="37">
         <f>COUNTIF(AG5:AG28,"Sim")+COUNTIF(AG5:AG28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AH31" s="37">
         <f>COUNTIF(AH5:AH28,"Sim")+COUNTIF(AH5:AH28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AI31" s="37">
         <f>COUNTIF(AI5:AI28,"Sim")+COUNTIF(AI5:AI28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AJ31" s="37">
         <f>COUNTIF(AJ5:AJ28,"Sim")+COUNTIF(AJ5:AJ28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK31" s="37">
         <f>COUNTIF(AK5:AK28,"Sim")+COUNTIF(AK5:AK28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL31" s="37">
         <f>COUNTIF(AL5:AL28,"Sim")+COUNTIF(AL5:AL28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AM31" s="37">
         <f>COUNTIF(AM5:AM28,"Sim")+COUNTIF(AM5:AM28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AN31" s="37">
         <f>COUNTIF(AN5:AN28,"Sim")+COUNTIF(AN5:AN28,"Não")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO31" s="37">
         <f>COUNTIF(AO5:AO28,"Sim")+COUNTIF(AO5:AO28,"Não")</f>
@@ -5576,211 +5530,211 @@
       </c>
       <c r="E32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Y32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Z32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AB32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AC32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AD32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AE32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AF32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AH32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AI32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AJ32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AM32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AN32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AP32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AQ32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AR32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AS32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AT32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AU32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AV32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AW32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AX32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AY32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AZ32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BA32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BB32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BC32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BD32" s="37">
         <f>COUNTA($B$5:$B$28)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
@@ -5903,35 +5857,35 @@
       </c>
       <c r="AG33" s="23">
         <f>IF(AG31=0,"",AG30/AG32)</f>
-        <v>0.555555555555556</v>
+        <v>0.5</v>
       </c>
       <c r="AH33" s="23">
         <f>IF(AH31=0,"",AH30/AH32)</f>
-        <v>0.888888888888889</v>
+        <v>0.875</v>
       </c>
       <c r="AI33" s="23">
         <f>IF(AI31=0,"",AI30/AI32)</f>
-        <v>0.888888888888889</v>
+        <v>0.75</v>
       </c>
       <c r="AJ33" s="23">
         <f>IF(AJ31=0,"",AJ30/AJ32)</f>
-        <v>0.888888888888889</v>
+        <v>1</v>
       </c>
       <c r="AK33" s="23">
         <f>IF(AK31=0,"",AK30/AK32)</f>
-        <v>0.888888888888889</v>
+        <v>0.75</v>
       </c>
       <c r="AL33" s="23">
         <f>IF(AL31=0,"",AL30/AL32)</f>
-        <v>0.777777777777778</v>
+        <v>0.875</v>
       </c>
       <c r="AM33" s="23">
         <f>IF(AM31=0,"",AM30/AM32)</f>
-        <v>0.777777777777778</v>
+        <v>0.875</v>
       </c>
       <c r="AN33" s="23">
         <f>IF(AN31=0,"",AN30/AN32)</f>
-        <v>0.888888888888889</v>
+        <v>0.875</v>
       </c>
       <c r="AO33" s="23">
         <f>IF(AO31=0,"",AO30/AO32)</f>
@@ -6118,35 +6072,35 @@
       </c>
       <c r="AG34" s="37">
         <f>SUMIF(AG5:AG28,"Sim",$C$5:$C$28)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AH34" s="37">
         <f>SUMIF(AH5:AH28,"Sim",$C$5:$C$28)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AI34" s="37">
         <f>SUMIF(AI5:AI28,"Sim",$C$5:$C$28)</f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AJ34" s="37">
         <f>SUMIF(AJ5:AJ28,"Sim",$C$5:$C$28)</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="AK34" s="37">
         <f>SUMIF(AK5:AK28,"Sim",$C$5:$C$28)</f>
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="AL34" s="37">
         <f>SUMIF(AL5:AL28,"Sim",$C$5:$C$28)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="AM34" s="37">
         <f>SUMIF(AM5:AM28,"Sim",$C$5:$C$28)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AN34" s="37">
         <f>SUMIF(AN5:AN28,"Sim",$C$5:$C$28)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AO34" s="37">
         <f>SUMIF(AO5:AO28,"Sim",$C$5:$C$28)</f>
@@ -6220,10 +6174,18 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Quem lança o caixa: a recepção lança o fechamento do dia na planilha 09 todo dia, no fechamento (planilha 04 · Checklist do dia). Na sexta a sócia só CONFERE os cinco fechamentos da semana contra o extrato — por isso a rotina de sexta diz "conferir", e não "lançar".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:BD28">

</xml_diff>